<commit_message>
changes of files d15N
</commit_message>
<xml_diff>
--- a/dataRESTICFOR/plot_charaterisation_RESTICFOR.xlsx
+++ b/dataRESTICFOR/plot_charaterisation_RESTICFOR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://creaf-my.sharepoint.com/personal/t_gimeno_creaf_uab_cat/Documents/terefi/repo/RESTICFOR/dataRESTICFOR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{0F1814C2-5E4F-42CC-AC2E-D92458D70243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16BC01E7-7C3B-443D-B799-FC4AF6C6BCCF}"/>
+  <xr:revisionPtr revIDLastSave="192" documentId="13_ncr:1_{0F1814C2-5E4F-42CC-AC2E-D92458D70243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C1A8949-9F83-4121-8A2B-30800A832F84}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="plot_id" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17270" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17272" uniqueCount="155">
   <si>
     <t>plotID</t>
   </si>
@@ -502,6 +502,12 @@
   <si>
     <t>HT,TEG, EM, IC</t>
   </si>
+  <si>
+    <t>sampling_radius_m</t>
+  </si>
+  <si>
+    <t>number_quarters_sampled</t>
+  </si>
 </sst>
 </file>
 
@@ -510,7 +516,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -581,6 +587,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -602,7 +615,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -620,6 +633,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -934,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48C1BCF0-F6AB-4E7E-B087-24C4BDC9548F}">
-  <dimension ref="A1:S31"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" customWidth="1"/>
@@ -955,7 +969,7 @@
     <col min="19" max="19" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -1013,8 +1027,14 @@
       <c r="S1" s="13" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="U1" s="17" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
@@ -1073,8 +1093,14 @@
       <c r="S2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T2" s="12">
+        <v>10</v>
+      </c>
+      <c r="U2" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1133,8 +1159,14 @@
       <c r="S3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T3" s="12">
+        <v>10</v>
+      </c>
+      <c r="U3" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1163,7 +1195,7 @@
         <v>26</v>
       </c>
       <c r="J4" s="9">
-        <v>46045</v>
+        <v>46318</v>
       </c>
       <c r="K4" s="10" t="s">
         <v>29</v>
@@ -1193,8 +1225,14 @@
       <c r="S4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T4" s="12">
+        <v>10</v>
+      </c>
+      <c r="U4" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
@@ -1253,8 +1291,14 @@
       <c r="S5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T5" s="12">
+        <v>10</v>
+      </c>
+      <c r="U5" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
@@ -1313,8 +1357,14 @@
       <c r="S6" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T6" s="12">
+        <v>10</v>
+      </c>
+      <c r="U6" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -1373,8 +1423,14 @@
       <c r="S7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T7" s="12">
+        <v>10</v>
+      </c>
+      <c r="U7" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1434,8 +1490,14 @@
       <c r="S8" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T8" s="12">
+        <v>10</v>
+      </c>
+      <c r="U8" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -1494,8 +1556,14 @@
       <c r="S9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T9" s="12">
+        <v>10</v>
+      </c>
+      <c r="U9" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1554,8 +1622,14 @@
       <c r="S10" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T10" s="12">
+        <v>10</v>
+      </c>
+      <c r="U10" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1614,8 +1688,14 @@
       <c r="S11" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T11" s="12">
+        <v>10</v>
+      </c>
+      <c r="U11" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1675,8 +1755,14 @@
       <c r="S12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T12" s="12">
+        <v>15</v>
+      </c>
+      <c r="U12" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -1736,8 +1822,14 @@
       <c r="S13" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T13" s="12">
+        <v>10</v>
+      </c>
+      <c r="U13" s="12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -1797,8 +1889,14 @@
       <c r="S14" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T14" s="12">
+        <v>10</v>
+      </c>
+      <c r="U14" s="12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -1858,8 +1956,14 @@
       <c r="S15" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T15" s="12">
+        <v>10</v>
+      </c>
+      <c r="U15" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -1918,8 +2022,14 @@
       <c r="S16" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T16" s="12">
+        <v>10</v>
+      </c>
+      <c r="U16" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>56</v>
       </c>
@@ -1978,8 +2088,14 @@
       <c r="S17" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T17" s="12">
+        <v>10</v>
+      </c>
+      <c r="U17" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>57</v>
       </c>
@@ -2039,8 +2155,14 @@
       <c r="S18" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T18" s="12">
+        <v>10</v>
+      </c>
+      <c r="U18" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -2099,8 +2221,14 @@
       <c r="S19" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T19" s="12">
+        <v>10</v>
+      </c>
+      <c r="U19" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -2159,8 +2287,14 @@
       <c r="S20" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T20" s="12">
+        <v>10</v>
+      </c>
+      <c r="U20" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -2219,8 +2353,14 @@
       <c r="S21" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T21" s="12">
+        <v>10</v>
+      </c>
+      <c r="U21" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>66</v>
       </c>
@@ -2250,7 +2390,7 @@
         <v>26</v>
       </c>
       <c r="J22" s="9">
-        <v>45788</v>
+        <v>45966</v>
       </c>
       <c r="K22" s="4" t="s">
         <v>49</v>
@@ -2280,8 +2420,14 @@
       <c r="S22" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T22" s="12">
+        <v>15</v>
+      </c>
+      <c r="U22" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>69</v>
       </c>
@@ -2341,8 +2487,14 @@
       <c r="S23" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T23" s="12">
+        <v>15</v>
+      </c>
+      <c r="U23" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>70</v>
       </c>
@@ -2402,8 +2554,14 @@
       <c r="S24" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T24" s="12">
+        <v>15</v>
+      </c>
+      <c r="U24" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -2463,8 +2621,14 @@
       <c r="S25" s="11" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T25" s="12">
+        <v>15</v>
+      </c>
+      <c r="U25" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>76</v>
       </c>
@@ -2524,8 +2688,14 @@
       <c r="S26" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T26" s="12">
+        <v>15</v>
+      </c>
+      <c r="U26" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -2584,8 +2754,14 @@
       <c r="S27" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T27" s="12">
+        <v>15</v>
+      </c>
+      <c r="U27" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -2644,8 +2820,14 @@
       <c r="S28" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T28" s="12">
+        <v>15</v>
+      </c>
+      <c r="U28" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>82</v>
       </c>
@@ -2705,8 +2887,14 @@
       <c r="S29" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T29" s="12">
+        <v>15</v>
+      </c>
+      <c r="U29" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>84</v>
       </c>
@@ -2766,8 +2954,14 @@
       <c r="S30" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T30" s="12">
+        <v>15</v>
+      </c>
+      <c r="U30" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>141</v>
       </c>
@@ -2825,6 +3019,12 @@
       </c>
       <c r="S31" t="s">
         <v>42</v>
+      </c>
+      <c r="T31" s="12">
+        <v>15</v>
+      </c>
+      <c r="U31" s="12">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>